<commit_message>
adding mutand v healthy comparison, evolution and orthologs and update gantt
</commit_message>
<xml_diff>
--- a/gant/live/gantt_live.xlsx
+++ b/gant/live/gantt_live.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="159">
   <si>
     <t xml:space="preserve">PROJECT TITLE</t>
   </si>
@@ -313,9 +313,6 @@
   </si>
   <si>
     <t xml:space="preserve">OMIM: gene-disease relationship</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pending</t>
   </si>
   <si>
     <t xml:space="preserve">Output: Notes on the gene and the phenotype</t>
@@ -590,7 +587,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -635,14 +632,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF8CBAD"/>
-        <bgColor rgb="FFFFE699"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFE699"/>
-        <bgColor rgb="FFF8CBAD"/>
+        <bgColor rgb="FFFFCC99"/>
       </patternFill>
     </fill>
     <fill>
@@ -769,7 +760,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -782,7 +773,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -878,7 +869,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -886,43 +889,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="11" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -980,7 +967,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFF8CBAD"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF2A78D6"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -2010,8 +1997,8 @@
         <f aca="false">NETWORKDAYS(D18,E18,Holidays!$A$2:$A$1000)</f>
         <v>5</v>
       </c>
-      <c r="I18" s="26" t="s">
-        <v>89</v>
+      <c r="I18" s="19" t="s">
+        <v>53</v>
       </c>
       <c r="J18" s="17"/>
       <c r="K18" s="17"/>
@@ -2039,15 +2026,15 @@
       <c r="AG18" s="17"/>
       <c r="AH18" s="17"/>
       <c r="AI18" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B19" s="17" t="s">
         <v>91</v>
-      </c>
-      <c r="B19" s="17" t="s">
-        <v>92</v>
       </c>
       <c r="C19" s="17" t="s">
         <v>65</v>
@@ -2097,15 +2084,15 @@
       <c r="AG19" s="17"/>
       <c r="AH19" s="17"/>
       <c r="AI19" s="21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="17" t="s">
         <v>94</v>
-      </c>
-      <c r="B20" s="17" t="s">
-        <v>95</v>
       </c>
       <c r="C20" s="17" t="s">
         <v>69</v>
@@ -2155,15 +2142,15 @@
       <c r="AG20" s="17"/>
       <c r="AH20" s="17"/>
       <c r="AI20" s="21" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B21" s="17" t="s">
         <v>97</v>
-      </c>
-      <c r="B21" s="17" t="s">
-        <v>98</v>
       </c>
       <c r="C21" s="17" t="s">
         <v>69</v>
@@ -2213,15 +2200,15 @@
       <c r="AG21" s="17"/>
       <c r="AH21" s="17"/>
       <c r="AI21" s="21" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="B22" s="17" t="s">
         <v>100</v>
-      </c>
-      <c r="B22" s="17" t="s">
-        <v>101</v>
       </c>
       <c r="C22" s="17" t="s">
         <v>82</v>
@@ -2240,8 +2227,8 @@
         <f aca="false">NETWORKDAYS(D22,E22,Holidays!$A$2:$A$1000)</f>
         <v>15</v>
       </c>
-      <c r="I22" s="27" t="s">
-        <v>102</v>
+      <c r="I22" s="26" t="s">
+        <v>101</v>
       </c>
       <c r="J22" s="24"/>
       <c r="K22" s="24"/>
@@ -2269,15 +2256,15 @@
       <c r="AG22" s="17"/>
       <c r="AH22" s="17"/>
       <c r="AI22" s="21" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>104</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>105</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="14" t="n">
@@ -2322,10 +2309,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B24" s="17" t="s">
         <v>106</v>
-      </c>
-      <c r="B24" s="17" t="s">
-        <v>107</v>
       </c>
       <c r="C24" s="17" t="s">
         <v>52</v>
@@ -2356,9 +2343,9 @@
       <c r="N24" s="17"/>
       <c r="O24" s="17"/>
       <c r="P24" s="20"/>
-      <c r="Q24" s="28"/>
-      <c r="R24" s="29"/>
-      <c r="S24" s="29"/>
+      <c r="Q24" s="27"/>
+      <c r="R24" s="28"/>
+      <c r="S24" s="28"/>
       <c r="T24" s="17"/>
       <c r="U24" s="20"/>
       <c r="V24" s="17"/>
@@ -2375,15 +2362,15 @@
       <c r="AG24" s="17"/>
       <c r="AH24" s="17"/>
       <c r="AI24" s="21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="B25" s="17" t="s">
         <v>109</v>
-      </c>
-      <c r="B25" s="17" t="s">
-        <v>110</v>
       </c>
       <c r="C25" s="17" t="s">
         <v>76</v>
@@ -2416,9 +2403,9 @@
       <c r="P25" s="20"/>
       <c r="Q25" s="20"/>
       <c r="R25" s="17"/>
-      <c r="S25" s="29"/>
-      <c r="T25" s="29"/>
-      <c r="U25" s="28"/>
+      <c r="S25" s="28"/>
+      <c r="T25" s="28"/>
+      <c r="U25" s="27"/>
       <c r="V25" s="17"/>
       <c r="W25" s="17"/>
       <c r="X25" s="20"/>
@@ -2433,18 +2420,18 @@
       <c r="AG25" s="17"/>
       <c r="AH25" s="17"/>
       <c r="AI25" s="21" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B26" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="C26" s="17" t="s">
         <v>113</v>
-      </c>
-      <c r="C26" s="17" t="s">
-        <v>114</v>
       </c>
       <c r="D26" s="18" t="n">
         <v>46308</v>
@@ -2455,13 +2442,15 @@
       <c r="F26" s="18" t="n">
         <v>46310</v>
       </c>
-      <c r="G26" s="17"/>
+      <c r="G26" s="18" t="n">
+        <v>46316</v>
+      </c>
       <c r="H26" s="17" t="n">
         <f aca="false">NETWORKDAYS(D26,E26,Holidays!$A$2:$A$1000)</f>
         <v>5</v>
       </c>
-      <c r="I26" s="27" t="s">
-        <v>102</v>
+      <c r="I26" s="19" t="s">
+        <v>53</v>
       </c>
       <c r="J26" s="17"/>
       <c r="K26" s="17"/>
@@ -2470,11 +2459,11 @@
       <c r="N26" s="17"/>
       <c r="O26" s="17"/>
       <c r="P26" s="20"/>
-      <c r="Q26" s="28"/>
-      <c r="R26" s="29"/>
-      <c r="S26" s="29"/>
-      <c r="T26" s="29"/>
-      <c r="U26" s="28"/>
+      <c r="Q26" s="27"/>
+      <c r="R26" s="28"/>
+      <c r="S26" s="28"/>
+      <c r="T26" s="28"/>
+      <c r="U26" s="27"/>
       <c r="V26" s="17"/>
       <c r="W26" s="17"/>
       <c r="X26" s="20"/>
@@ -2489,15 +2478,15 @@
       <c r="AG26" s="17"/>
       <c r="AH26" s="17"/>
       <c r="AI26" s="21" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="B27" s="17" t="s">
         <v>116</v>
-      </c>
-      <c r="B27" s="17" t="s">
-        <v>117</v>
       </c>
       <c r="C27" s="17" t="s">
         <v>61</v>
@@ -2514,8 +2503,8 @@
         <f aca="false">NETWORKDAYS(D27,E27,Holidays!$A$2:$A$1000)</f>
         <v>3</v>
       </c>
-      <c r="I27" s="30" t="s">
-        <v>118</v>
+      <c r="I27" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J27" s="17"/>
       <c r="K27" s="17"/>
@@ -2529,9 +2518,9 @@
       <c r="S27" s="17"/>
       <c r="T27" s="17"/>
       <c r="U27" s="20"/>
-      <c r="V27" s="29"/>
-      <c r="W27" s="29"/>
-      <c r="X27" s="28"/>
+      <c r="V27" s="28"/>
+      <c r="W27" s="28"/>
+      <c r="X27" s="27"/>
       <c r="Y27" s="17"/>
       <c r="Z27" s="20"/>
       <c r="AA27" s="17"/>
@@ -2543,18 +2532,18 @@
       <c r="AG27" s="17"/>
       <c r="AH27" s="17"/>
       <c r="AI27" s="21" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="B28" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="B28" s="17" t="s">
-        <v>121</v>
-      </c>
       <c r="C28" s="17" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D28" s="18" t="n">
         <v>46308</v>
@@ -2565,13 +2554,15 @@
       <c r="F28" s="18" t="n">
         <v>46310</v>
       </c>
-      <c r="G28" s="17"/>
+      <c r="G28" s="18" t="n">
+        <v>46316</v>
+      </c>
       <c r="H28" s="17" t="n">
         <f aca="false">NETWORKDAYS(D28,E28,Holidays!$A$2:$A$1000)</f>
         <v>5</v>
       </c>
-      <c r="I28" s="27" t="s">
-        <v>102</v>
+      <c r="I28" s="19" t="s">
+        <v>53</v>
       </c>
       <c r="J28" s="17"/>
       <c r="K28" s="17"/>
@@ -2580,11 +2571,11 @@
       <c r="N28" s="17"/>
       <c r="O28" s="17"/>
       <c r="P28" s="20"/>
-      <c r="Q28" s="28"/>
-      <c r="R28" s="29"/>
-      <c r="S28" s="29"/>
-      <c r="T28" s="29"/>
-      <c r="U28" s="28"/>
+      <c r="Q28" s="27"/>
+      <c r="R28" s="28"/>
+      <c r="S28" s="28"/>
+      <c r="T28" s="28"/>
+      <c r="U28" s="27"/>
       <c r="V28" s="17"/>
       <c r="W28" s="17"/>
       <c r="X28" s="20"/>
@@ -2599,15 +2590,15 @@
       <c r="AG28" s="17"/>
       <c r="AH28" s="17"/>
       <c r="AI28" s="21" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="B29" s="17" t="s">
         <v>123</v>
-      </c>
-      <c r="B29" s="17" t="s">
-        <v>124</v>
       </c>
       <c r="C29" s="17" t="s">
         <v>65</v>
@@ -2624,8 +2615,8 @@
         <f aca="false">NETWORKDAYS(D29,E29,Holidays!$A$2:$A$1000)</f>
         <v>3</v>
       </c>
-      <c r="I29" s="30" t="s">
-        <v>118</v>
+      <c r="I29" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J29" s="17"/>
       <c r="K29" s="17"/>
@@ -2639,9 +2630,9 @@
       <c r="S29" s="17"/>
       <c r="T29" s="17"/>
       <c r="U29" s="20"/>
-      <c r="V29" s="29"/>
-      <c r="W29" s="29"/>
-      <c r="X29" s="28"/>
+      <c r="V29" s="28"/>
+      <c r="W29" s="28"/>
+      <c r="X29" s="27"/>
       <c r="Y29" s="17"/>
       <c r="Z29" s="20"/>
       <c r="AA29" s="17"/>
@@ -2653,15 +2644,15 @@
       <c r="AG29" s="17"/>
       <c r="AH29" s="17"/>
       <c r="AI29" s="21" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="B30" s="12" t="s">
         <v>126</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>127</v>
       </c>
       <c r="C30" s="13"/>
       <c r="D30" s="14" t="n">
@@ -2706,10 +2697,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="B31" s="17" t="s">
         <v>128</v>
-      </c>
-      <c r="B31" s="17" t="s">
-        <v>129</v>
       </c>
       <c r="C31" s="17" t="s">
         <v>57</v>
@@ -2726,8 +2717,8 @@
         <f aca="false">NETWORKDAYS(D31,E31,Holidays!$A$2:$A$1000)</f>
         <v>1</v>
       </c>
-      <c r="I31" s="30" t="s">
-        <v>118</v>
+      <c r="I31" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J31" s="17"/>
       <c r="K31" s="17"/>
@@ -2741,7 +2732,7 @@
       <c r="S31" s="17"/>
       <c r="T31" s="17"/>
       <c r="U31" s="20"/>
-      <c r="V31" s="31"/>
+      <c r="V31" s="30"/>
       <c r="W31" s="17"/>
       <c r="X31" s="20"/>
       <c r="Y31" s="17"/>
@@ -2758,10 +2749,10 @@
     </row>
     <row r="32" customFormat="false" ht="15.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="16" t="s">
+        <v>129</v>
+      </c>
+      <c r="B32" s="17" t="s">
         <v>130</v>
-      </c>
-      <c r="B32" s="17" t="s">
-        <v>131</v>
       </c>
       <c r="C32" s="17" t="s">
         <v>82</v>
@@ -2778,8 +2769,8 @@
         <f aca="false">NETWORKDAYS(D32,E32,Holidays!$A$2:$A$1000)</f>
         <v>1</v>
       </c>
-      <c r="I32" s="30" t="s">
-        <v>118</v>
+      <c r="I32" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J32" s="17"/>
       <c r="K32" s="17"/>
@@ -2791,7 +2782,7 @@
       <c r="Q32" s="20"/>
       <c r="R32" s="17"/>
       <c r="S32" s="17"/>
-      <c r="T32" s="31"/>
+      <c r="T32" s="30"/>
       <c r="U32" s="20"/>
       <c r="V32" s="17"/>
       <c r="W32" s="17"/>
@@ -2807,15 +2798,15 @@
       <c r="AG32" s="17"/>
       <c r="AH32" s="17"/>
       <c r="AI32" s="21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="B33" s="17" t="s">
         <v>133</v>
-      </c>
-      <c r="B33" s="17" t="s">
-        <v>134</v>
       </c>
       <c r="C33" s="17" t="s">
         <v>82</v>
@@ -2832,8 +2823,8 @@
         <f aca="false">NETWORKDAYS(D33,E33,Holidays!$A$2:$A$1000)</f>
         <v>4</v>
       </c>
-      <c r="I33" s="30" t="s">
-        <v>118</v>
+      <c r="I33" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J33" s="17"/>
       <c r="K33" s="17"/>
@@ -2846,10 +2837,10 @@
       <c r="R33" s="17"/>
       <c r="S33" s="17"/>
       <c r="T33" s="17"/>
-      <c r="U33" s="32"/>
-      <c r="V33" s="31"/>
-      <c r="W33" s="31"/>
-      <c r="X33" s="32"/>
+      <c r="U33" s="31"/>
+      <c r="V33" s="30"/>
+      <c r="W33" s="30"/>
+      <c r="X33" s="31"/>
       <c r="Y33" s="17"/>
       <c r="Z33" s="20"/>
       <c r="AA33" s="17"/>
@@ -2864,13 +2855,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="B34" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="B34" s="17" t="s">
-        <v>136</v>
-      </c>
       <c r="C34" s="17" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D34" s="18" t="n">
         <v>46315</v>
@@ -2884,8 +2875,8 @@
         <f aca="false">NETWORKDAYS(D34,E34,Holidays!$A$2:$A$1000)</f>
         <v>3</v>
       </c>
-      <c r="I34" s="30" t="s">
-        <v>118</v>
+      <c r="I34" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J34" s="17"/>
       <c r="K34" s="17"/>
@@ -2899,9 +2890,9 @@
       <c r="S34" s="17"/>
       <c r="T34" s="17"/>
       <c r="U34" s="20"/>
-      <c r="V34" s="31"/>
-      <c r="W34" s="31"/>
-      <c r="X34" s="32"/>
+      <c r="V34" s="30"/>
+      <c r="W34" s="30"/>
+      <c r="X34" s="31"/>
       <c r="Y34" s="17"/>
       <c r="Z34" s="20"/>
       <c r="AA34" s="17"/>
@@ -2916,10 +2907,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16" t="s">
+        <v>136</v>
+      </c>
+      <c r="B35" s="17" t="s">
         <v>137</v>
-      </c>
-      <c r="B35" s="17" t="s">
-        <v>138</v>
       </c>
       <c r="C35" s="17" t="s">
         <v>76</v>
@@ -2936,8 +2927,8 @@
         <f aca="false">NETWORKDAYS(D35,E35,Holidays!$A$2:$A$1000)</f>
         <v>3</v>
       </c>
-      <c r="I35" s="30" t="s">
-        <v>118</v>
+      <c r="I35" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J35" s="17"/>
       <c r="K35" s="17"/>
@@ -2951,9 +2942,9 @@
       <c r="S35" s="17"/>
       <c r="T35" s="17"/>
       <c r="U35" s="20"/>
-      <c r="V35" s="31"/>
-      <c r="W35" s="31"/>
-      <c r="X35" s="32"/>
+      <c r="V35" s="30"/>
+      <c r="W35" s="30"/>
+      <c r="X35" s="31"/>
       <c r="Y35" s="17"/>
       <c r="Z35" s="20"/>
       <c r="AA35" s="17"/>
@@ -2968,10 +2959,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="B36" s="17" t="s">
         <v>139</v>
-      </c>
-      <c r="B36" s="17" t="s">
-        <v>140</v>
       </c>
       <c r="C36" s="17" t="s">
         <v>65</v>
@@ -2988,8 +2979,8 @@
         <f aca="false">NETWORKDAYS(D36,E36,Holidays!$A$2:$A$1000)</f>
         <v>3</v>
       </c>
-      <c r="I36" s="30" t="s">
-        <v>118</v>
+      <c r="I36" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J36" s="17"/>
       <c r="K36" s="17"/>
@@ -3003,9 +2994,9 @@
       <c r="S36" s="17"/>
       <c r="T36" s="17"/>
       <c r="U36" s="20"/>
-      <c r="V36" s="31"/>
-      <c r="W36" s="31"/>
-      <c r="X36" s="32"/>
+      <c r="V36" s="30"/>
+      <c r="W36" s="30"/>
+      <c r="X36" s="31"/>
       <c r="Y36" s="17"/>
       <c r="Z36" s="20"/>
       <c r="AA36" s="17"/>
@@ -3020,10 +3011,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="B37" s="17" t="s">
         <v>141</v>
-      </c>
-      <c r="B37" s="17" t="s">
-        <v>142</v>
       </c>
       <c r="C37" s="17" t="s">
         <v>69</v>
@@ -3040,8 +3031,8 @@
         <f aca="false">NETWORKDAYS(D37,E37,Holidays!$A$2:$A$1000)</f>
         <v>2</v>
       </c>
-      <c r="I37" s="30" t="s">
-        <v>118</v>
+      <c r="I37" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J37" s="17"/>
       <c r="K37" s="17"/>
@@ -3057,8 +3048,8 @@
       <c r="U37" s="20"/>
       <c r="V37" s="17"/>
       <c r="W37" s="17"/>
-      <c r="X37" s="32"/>
-      <c r="Y37" s="31"/>
+      <c r="X37" s="31"/>
+      <c r="Y37" s="30"/>
       <c r="Z37" s="20"/>
       <c r="AA37" s="17"/>
       <c r="AB37" s="17"/>
@@ -3072,10 +3063,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="B38" s="17" t="s">
         <v>143</v>
-      </c>
-      <c r="B38" s="17" t="s">
-        <v>144</v>
       </c>
       <c r="C38" s="17" t="s">
         <v>57</v>
@@ -3092,8 +3083,8 @@
         <f aca="false">NETWORKDAYS(D38,E38,Holidays!$A$2:$A$1000)</f>
         <v>1</v>
       </c>
-      <c r="I38" s="30" t="s">
-        <v>118</v>
+      <c r="I38" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J38" s="17"/>
       <c r="K38" s="17"/>
@@ -3110,7 +3101,7 @@
       <c r="V38" s="17"/>
       <c r="W38" s="17"/>
       <c r="X38" s="20"/>
-      <c r="Y38" s="31"/>
+      <c r="Y38" s="30"/>
       <c r="Z38" s="20"/>
       <c r="AA38" s="17"/>
       <c r="AB38" s="17"/>
@@ -3124,10 +3115,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="B39" s="17" t="s">
         <v>145</v>
-      </c>
-      <c r="B39" s="17" t="s">
-        <v>146</v>
       </c>
       <c r="C39" s="17" t="s">
         <v>65</v>
@@ -3144,8 +3135,8 @@
         <f aca="false">NETWORKDAYS(D39,E39,Holidays!$A$2:$A$1000)</f>
         <v>1</v>
       </c>
-      <c r="I39" s="30" t="s">
-        <v>118</v>
+      <c r="I39" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J39" s="17"/>
       <c r="K39" s="17"/>
@@ -3163,7 +3154,7 @@
       <c r="W39" s="17"/>
       <c r="X39" s="20"/>
       <c r="Y39" s="17"/>
-      <c r="Z39" s="32"/>
+      <c r="Z39" s="31"/>
       <c r="AA39" s="17"/>
       <c r="AB39" s="17"/>
       <c r="AC39" s="17"/>
@@ -3176,10 +3167,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="B40" s="12" t="s">
         <v>147</v>
-      </c>
-      <c r="B40" s="12" t="s">
-        <v>148</v>
       </c>
       <c r="C40" s="13"/>
       <c r="D40" s="14" t="n">
@@ -3224,10 +3215,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="B41" s="17" t="s">
         <v>149</v>
-      </c>
-      <c r="B41" s="17" t="s">
-        <v>150</v>
       </c>
       <c r="C41" s="17" t="s">
         <v>57</v>
@@ -3244,8 +3235,8 @@
         <f aca="false">NETWORKDAYS(D41,E41,Holidays!$A$2:$A$1000)</f>
         <v>3</v>
       </c>
-      <c r="I41" s="30" t="s">
-        <v>118</v>
+      <c r="I41" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J41" s="17"/>
       <c r="K41" s="17"/>
@@ -3264,9 +3255,9 @@
       <c r="X41" s="20"/>
       <c r="Y41" s="17"/>
       <c r="Z41" s="20"/>
-      <c r="AA41" s="33"/>
-      <c r="AB41" s="33"/>
-      <c r="AC41" s="33"/>
+      <c r="AA41" s="32"/>
+      <c r="AB41" s="32"/>
+      <c r="AC41" s="32"/>
       <c r="AD41" s="17"/>
       <c r="AE41" s="17"/>
       <c r="AF41" s="17"/>
@@ -3276,10 +3267,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="B42" s="17" t="s">
         <v>151</v>
-      </c>
-      <c r="B42" s="17" t="s">
-        <v>152</v>
       </c>
       <c r="C42" s="17" t="s">
         <v>69</v>
@@ -3296,8 +3287,8 @@
         <f aca="false">NETWORKDAYS(D42,E42,Holidays!$A$2:$A$1000)</f>
         <v>1</v>
       </c>
-      <c r="I42" s="30" t="s">
-        <v>118</v>
+      <c r="I42" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J42" s="17"/>
       <c r="K42" s="17"/>
@@ -3319,7 +3310,7 @@
       <c r="AA42" s="17"/>
       <c r="AB42" s="17"/>
       <c r="AC42" s="17"/>
-      <c r="AD42" s="33"/>
+      <c r="AD42" s="32"/>
       <c r="AE42" s="17"/>
       <c r="AF42" s="17"/>
       <c r="AG42" s="17"/>
@@ -3328,10 +3319,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="B43" s="17" t="s">
         <v>153</v>
-      </c>
-      <c r="B43" s="17" t="s">
-        <v>154</v>
       </c>
       <c r="C43" s="17" t="s">
         <v>57</v>
@@ -3348,8 +3339,8 @@
         <f aca="false">NETWORKDAYS(D43,E43,Holidays!$A$2:$A$1000)</f>
         <v>2</v>
       </c>
-      <c r="I43" s="30" t="s">
-        <v>118</v>
+      <c r="I43" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J43" s="17"/>
       <c r="K43" s="17"/>
@@ -3373,17 +3364,17 @@
       <c r="AC43" s="17"/>
       <c r="AD43" s="17"/>
       <c r="AE43" s="17"/>
-      <c r="AF43" s="33"/>
-      <c r="AG43" s="33"/>
+      <c r="AF43" s="32"/>
+      <c r="AG43" s="32"/>
       <c r="AH43" s="17"/>
       <c r="AI43" s="21"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="B44" s="17" t="s">
         <v>155</v>
-      </c>
-      <c r="B44" s="17" t="s">
-        <v>156</v>
       </c>
       <c r="C44" s="17" t="s">
         <v>57</v>
@@ -3400,8 +3391,8 @@
         <f aca="false">NETWORKDAYS(D44,E44,Holidays!$A$2:$A$1000)</f>
         <v>1</v>
       </c>
-      <c r="I44" s="30" t="s">
-        <v>118</v>
+      <c r="I44" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J44" s="17"/>
       <c r="K44" s="17"/>
@@ -3427,64 +3418,64 @@
       <c r="AE44" s="17"/>
       <c r="AF44" s="17"/>
       <c r="AG44" s="17"/>
-      <c r="AH44" s="33"/>
+      <c r="AH44" s="32"/>
       <c r="AI44" s="21"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M45" s="34"/>
-      <c r="P45" s="34"/>
-      <c r="Q45" s="34"/>
-      <c r="U45" s="34"/>
-      <c r="X45" s="34"/>
-      <c r="Z45" s="34"/>
+      <c r="M45" s="33"/>
+      <c r="P45" s="33"/>
+      <c r="Q45" s="33"/>
+      <c r="U45" s="33"/>
+      <c r="X45" s="33"/>
+      <c r="Z45" s="33"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="35" t="s">
+      <c r="A46" s="34" t="s">
+        <v>156</v>
+      </c>
+      <c r="B46" s="34" t="s">
         <v>157</v>
       </c>
-      <c r="B46" s="35" t="s">
-        <v>158</v>
-      </c>
-      <c r="C46" s="36"/>
-      <c r="D46" s="37" t="n">
+      <c r="C46" s="35"/>
+      <c r="D46" s="36" t="n">
         <v>46282</v>
       </c>
-      <c r="E46" s="37" t="n">
+      <c r="E46" s="36" t="n">
         <v>46331</v>
       </c>
-      <c r="F46" s="36"/>
-      <c r="G46" s="36"/>
-      <c r="H46" s="35" t="n">
+      <c r="F46" s="35"/>
+      <c r="G46" s="35"/>
+      <c r="H46" s="34" t="n">
         <f aca="false">NETWORKDAYS(D46,E46,Holidays!$A$2:$A$1000)</f>
         <v>34</v>
       </c>
-      <c r="I46" s="36"/>
-      <c r="J46" s="36"/>
-      <c r="K46" s="36"/>
-      <c r="L46" s="36"/>
-      <c r="M46" s="38"/>
-      <c r="N46" s="36"/>
-      <c r="O46" s="36"/>
-      <c r="P46" s="38"/>
-      <c r="Q46" s="38"/>
-      <c r="R46" s="36"/>
-      <c r="S46" s="36"/>
-      <c r="T46" s="36"/>
-      <c r="U46" s="38"/>
-      <c r="V46" s="36"/>
-      <c r="W46" s="36"/>
-      <c r="X46" s="38"/>
-      <c r="Y46" s="36"/>
-      <c r="Z46" s="38"/>
-      <c r="AA46" s="36"/>
-      <c r="AB46" s="36"/>
-      <c r="AC46" s="36"/>
-      <c r="AD46" s="36"/>
-      <c r="AE46" s="36"/>
-      <c r="AF46" s="36"/>
-      <c r="AG46" s="36"/>
-      <c r="AH46" s="36"/>
-      <c r="AI46" s="36"/>
+      <c r="I46" s="35"/>
+      <c r="J46" s="35"/>
+      <c r="K46" s="35"/>
+      <c r="L46" s="35"/>
+      <c r="M46" s="37"/>
+      <c r="N46" s="35"/>
+      <c r="O46" s="35"/>
+      <c r="P46" s="37"/>
+      <c r="Q46" s="37"/>
+      <c r="R46" s="35"/>
+      <c r="S46" s="35"/>
+      <c r="T46" s="35"/>
+      <c r="U46" s="37"/>
+      <c r="V46" s="35"/>
+      <c r="W46" s="35"/>
+      <c r="X46" s="37"/>
+      <c r="Y46" s="35"/>
+      <c r="Z46" s="37"/>
+      <c r="AA46" s="35"/>
+      <c r="AB46" s="35"/>
+      <c r="AC46" s="35"/>
+      <c r="AD46" s="35"/>
+      <c r="AE46" s="35"/>
+      <c r="AF46" s="35"/>
+      <c r="AG46" s="35"/>
+      <c r="AH46" s="35"/>
+      <c r="AI46" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -3525,26 +3516,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="39" t="n">
+      <c r="A2" s="38" t="n">
         <v>46276</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="39" t="n">
+      <c r="A3" s="38" t="n">
         <v>46289</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="39" t="n">
+      <c r="A4" s="38" t="n">
         <v>46307</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="39" t="n">
+      <c r="A5" s="38" t="n">
         <v>46364</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update FASTA files and gantt chart, upload methodology_v1
</commit_message>
<xml_diff>
--- a/gant/live/gantt_live.xlsx
+++ b/gant/live/gantt_live.xlsx
@@ -399,25 +399,25 @@
     <t xml:space="preserve">Figures</t>
   </si>
   <si>
+    <t xml:space="preserve">Output: Figures in figures/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evolutionary and homolog interpretation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Output: Interpretation notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limitations of each analysis</t>
+  </si>
+  <si>
     <t xml:space="preserve">Backlog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Output: Figures in figures/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evolutionary and homolog interpretation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Output: Interpretation notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Limitations of each analysis</t>
   </si>
   <si>
     <t xml:space="preserve">Output: Limitations summary (to be integrated into the Discussion section)</t>
@@ -2497,14 +2497,16 @@
       <c r="E27" s="18" t="n">
         <v>46317</v>
       </c>
-      <c r="F27" s="17"/>
+      <c r="F27" s="18" t="n">
+        <v>46317</v>
+      </c>
       <c r="G27" s="17"/>
       <c r="H27" s="17" t="n">
         <f aca="false">NETWORKDAYS(D27,E27,Holidays!$A$2:$A$1000)</f>
         <v>3</v>
       </c>
-      <c r="I27" s="29" t="s">
-        <v>117</v>
+      <c r="I27" s="26" t="s">
+        <v>101</v>
       </c>
       <c r="J27" s="17"/>
       <c r="K27" s="17"/>
@@ -2532,15 +2534,15 @@
       <c r="AG27" s="17"/>
       <c r="AH27" s="17"/>
       <c r="AI27" s="21" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="B28" s="17" t="s">
         <v>119</v>
-      </c>
-      <c r="B28" s="17" t="s">
-        <v>120</v>
       </c>
       <c r="C28" s="17" t="s">
         <v>113</v>
@@ -2590,15 +2592,15 @@
       <c r="AG28" s="17"/>
       <c r="AH28" s="17"/>
       <c r="AI28" s="21" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="B29" s="17" t="s">
         <v>122</v>
-      </c>
-      <c r="B29" s="17" t="s">
-        <v>123</v>
       </c>
       <c r="C29" s="17" t="s">
         <v>65</v>
@@ -2616,7 +2618,7 @@
         <v>3</v>
       </c>
       <c r="I29" s="29" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="J29" s="17"/>
       <c r="K29" s="17"/>
@@ -2718,7 +2720,7 @@
         <v>1</v>
       </c>
       <c r="I31" s="29" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="J31" s="17"/>
       <c r="K31" s="17"/>
@@ -2770,7 +2772,7 @@
         <v>1</v>
       </c>
       <c r="I32" s="29" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="J32" s="17"/>
       <c r="K32" s="17"/>
@@ -2824,7 +2826,7 @@
         <v>4</v>
       </c>
       <c r="I33" s="29" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="J33" s="17"/>
       <c r="K33" s="17"/>
@@ -2869,14 +2871,16 @@
       <c r="E34" s="18" t="n">
         <v>46317</v>
       </c>
-      <c r="F34" s="17"/>
+      <c r="F34" s="18" t="n">
+        <v>46316</v>
+      </c>
       <c r="G34" s="17"/>
       <c r="H34" s="17" t="n">
         <f aca="false">NETWORKDAYS(D34,E34,Holidays!$A$2:$A$1000)</f>
         <v>3</v>
       </c>
-      <c r="I34" s="29" t="s">
-        <v>117</v>
+      <c r="I34" s="26" t="s">
+        <v>101</v>
       </c>
       <c r="J34" s="17"/>
       <c r="K34" s="17"/>
@@ -2928,7 +2932,7 @@
         <v>3</v>
       </c>
       <c r="I35" s="29" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="J35" s="17"/>
       <c r="K35" s="17"/>
@@ -2980,7 +2984,7 @@
         <v>3</v>
       </c>
       <c r="I36" s="29" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="J36" s="17"/>
       <c r="K36" s="17"/>
@@ -3032,7 +3036,7 @@
         <v>2</v>
       </c>
       <c r="I37" s="29" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="J37" s="17"/>
       <c r="K37" s="17"/>
@@ -3084,7 +3088,7 @@
         <v>1</v>
       </c>
       <c r="I38" s="29" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="J38" s="17"/>
       <c r="K38" s="17"/>
@@ -3136,7 +3140,7 @@
         <v>1</v>
       </c>
       <c r="I39" s="29" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="J39" s="17"/>
       <c r="K39" s="17"/>
@@ -3236,7 +3240,7 @@
         <v>3</v>
       </c>
       <c r="I41" s="29" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="J41" s="17"/>
       <c r="K41" s="17"/>
@@ -3288,7 +3292,7 @@
         <v>1</v>
       </c>
       <c r="I42" s="29" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="J42" s="17"/>
       <c r="K42" s="17"/>
@@ -3340,7 +3344,7 @@
         <v>2</v>
       </c>
       <c r="I43" s="29" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="J43" s="17"/>
       <c r="K43" s="17"/>
@@ -3392,7 +3396,7 @@
         <v>1</v>
       </c>
       <c r="I44" s="29" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="J44" s="17"/>
       <c r="K44" s="17"/>

</xml_diff>